<commit_message>
Atualizando simulado e adicionando link formulário sprint 3
</commit_message>
<xml_diff>
--- a/projeto3/2023.1/sprint2/sprint2_medias.xlsx
+++ b/projeto3/2023.1/sprint2/sprint2_medias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,17 +491,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FERNANDO GIUSEPPE AVILA BELTRAMO</t>
+          <t>Gustavo Eliziario Stevenson de Oliveira</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F2" t="n">
         <v>3</v>
@@ -513,16 +513,16 @@
         <v>3</v>
       </c>
       <c r="I2" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="3">
@@ -531,7 +531,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ERIC ANDREI LIMA POSSATO</t>
+          <t>RODRIGO PAOLIELLO DE MEDEIROS</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -571,17 +571,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GUILHERME DOS SANTOS MARTINS</t>
+          <t>MATHEUS RAFFAELLE NERY CASTELLUCCI</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>3.333333333333333</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>3.333333333333333</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>3</v>
@@ -593,16 +593,16 @@
         <v>3</v>
       </c>
       <c r="I4" t="n">
-        <v>3.222222222222223</v>
+        <v>3</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.3333333333333335</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3333333333333335</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -611,17 +611,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PEDRO PAULO MORENO CAMARGO</t>
+          <t>LUCA MIZRAHI</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F5" t="n">
         <v>3</v>
@@ -633,16 +633,16 @@
         <v>3</v>
       </c>
       <c r="I5" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="6">
@@ -651,7 +651,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ANDRÉ CORRÊA SANTOS</t>
+          <t>JOÃO PEDRO RODRIGUES SANTOS</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -691,38 +691,38 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ANTÔNIO AMARAL EGYDIO MARTINS</t>
+          <t>ALBERTO MARTINS PEREIRA CARRERA</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3.666666666666667</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>3.666666666666667</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>3.666666666666667</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>3</v>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H7" t="n">
         <v>3</v>
       </c>
       <c r="I7" t="n">
-        <v>3.666666666666667</v>
+        <v>3</v>
       </c>
       <c r="J7" t="n">
-        <v>0.6666666666666665</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.3333333333333335</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6666666666666665</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -731,17 +731,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GIOVANA CASSONI ANDRADE</t>
+          <t>DOUGLAS PABLO</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>3.333333333333333</v>
+        <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>3.333333333333333</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
         <v>3</v>
@@ -753,16 +753,16 @@
         <v>3</v>
       </c>
       <c r="I8" t="n">
-        <v>3.222222222222223</v>
+        <v>3</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0.3333333333333335</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>0.3333333333333335</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -771,38 +771,38 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ENZO BOZELLI</t>
+          <t>BRUNO MARQUES LI VOLSI FALCAO</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>3</v>
       </c>
       <c r="G9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I9" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="J9" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5</v>
+        <v>-1</v>
       </c>
       <c r="L9" t="n">
-        <v>0.5</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="10">
@@ -811,38 +811,38 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RODRIGO ANCIÃES PATELLI</t>
+          <t>GABRIEL MENDONÇA DE MELLO HERMIDA</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10" t="n">
-        <v>3.333333333333333</v>
+        <v>4</v>
       </c>
       <c r="J10" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -851,29 +851,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>VINICIUS MATHEUS MORALES</t>
+          <t>ALEXANDRE RODRIGUES SANTAROSSA</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -891,38 +891,38 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>VICTOR LUIS GAMA DE ASSIS</t>
+          <t>KEVIN NAGAYUKI SHINOHARA</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3.333333333333333</v>
+        <v>3.666666666666667</v>
       </c>
       <c r="D12" t="n">
-        <v>3.333333333333333</v>
+        <v>3.666666666666667</v>
       </c>
       <c r="E12" t="n">
         <v>3.666666666666667</v>
       </c>
       <c r="F12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I12" t="n">
-        <v>3.444444444444445</v>
+        <v>3.666666666666667</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.6666666666666665</v>
+        <v>0.6666666666666665</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.6666666666666665</v>
+        <v>0.6666666666666665</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.3333333333333335</v>
+        <v>0.6666666666666665</v>
       </c>
     </row>
     <row r="13">
@@ -931,17 +931,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ARTHUR MARTINS DE SOUZA BARRETO</t>
+          <t>PEDRO TOLEDO PIZA CIVITA</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>3.333333333333333</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
         <v>4</v>
@@ -953,16 +953,16 @@
         <v>4</v>
       </c>
       <c r="I13" t="n">
-        <v>3.111111111111111</v>
+        <v>4</v>
       </c>
       <c r="J13" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.6666666666666665</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -971,38 +971,38 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LUCAS GURGEL</t>
+          <t>CAIO ORTEGA BÔA</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3.666666666666667</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>3.666666666666667</v>
+        <v>4</v>
       </c>
       <c r="E14" t="n">
         <v>4</v>
       </c>
       <c r="F14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I14" t="n">
-        <v>3.777777777777777</v>
+        <v>4</v>
       </c>
       <c r="J14" t="n">
-        <v>0.6666666666666665</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0.6666666666666665</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1011,32 +1011,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>LINCOLN RODRIGO PEREIRA MELO</t>
+          <t>ARTHUR MOREIRA TAMM</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I15" t="n">
-        <v>3.166666666666667</v>
+        <v>4</v>
       </c>
       <c r="J15" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DOM RUAN SUZANO FIGUEIRA DA SILVA</t>
+          <t>LUANA WILNER ABRAMOFF</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1091,29 +1091,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HUDSON MONTEIRO</t>
+          <t>RAFAEL PASCARELLI NICCHERI</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1131,29 +1131,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>JOÃO GABRIEL VALENTIM ROCHA</t>
+          <t>JOÃO ANTÔNIO GOMES GARCIA</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1171,17 +1171,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MURILO PRADO WEYNE</t>
+          <t>PEDRO AUGUSTO GEVE DE MORAES LACERDA</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3.333333333333333</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>3.666666666666667</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>3.333333333333333</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
         <v>3</v>
@@ -1193,16 +1193,16 @@
         <v>3</v>
       </c>
       <c r="I19" t="n">
-        <v>3.444444444444445</v>
+        <v>3</v>
       </c>
       <c r="J19" t="n">
-        <v>0.3333333333333335</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>0.6666666666666665</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>0.3333333333333335</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAIO RIBEIRO DE PAULA</t>
+          <t>PEDRO GOMES DE SÁ DRUMOND</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1251,17 +1251,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ARIEL TAMEZGUI LEVENTHAL</t>
+          <t>BRUNA LIMA MEINBERG</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3.333333333333333</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>3.666666666666667</v>
+        <v>4</v>
       </c>
       <c r="E21" t="n">
-        <v>3.333333333333333</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
         <v>4</v>
@@ -1273,16 +1273,16 @@
         <v>4</v>
       </c>
       <c r="I21" t="n">
-        <v>3.444444444444445</v>
+        <v>4</v>
       </c>
       <c r="J21" t="n">
-        <v>-0.6666666666666665</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>-0.3333333333333335</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>-0.6666666666666665</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1291,29 +1291,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PEDRO CLIQUET DO AMARAL</t>
+          <t>PEDRO HENRIQUE RIZO COLPAS</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ANDRÉ BRITO</t>
+          <t>GUSTAVO MENDES DA SILVA</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1350,7 +1350,7 @@
         <v>3</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I23" t="n">
         <v>3.666666666666667</v>
@@ -1362,7 +1362,7 @@
         <v>0.6666666666666665</v>
       </c>
       <c r="L23" t="n">
-        <v>-0.3333333333333335</v>
+        <v>0.6666666666666665</v>
       </c>
     </row>
     <row r="24">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ARTHUR CISOTTO MACHADO</t>
+          <t>GABRIELA KATSURAYAMA</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1381,7 +1381,7 @@
         <v>3.333333333333333</v>
       </c>
       <c r="E24" t="n">
-        <v>3.666666666666667</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="F24" t="n">
         <v>4</v>
@@ -1393,7 +1393,7 @@
         <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>3.444444444444445</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="J24" t="n">
         <v>-0.6666666666666665</v>
@@ -1402,7 +1402,7 @@
         <v>-0.6666666666666665</v>
       </c>
       <c r="L24" t="n">
-        <v>-0.3333333333333335</v>
+        <v>-0.6666666666666665</v>
       </c>
     </row>
     <row r="25">
@@ -1411,38 +1411,38 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MARLON SILVA PEREIRA</t>
+          <t>NICOLAS ENZO YASSUDA</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3.666666666666667</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="D25" t="n">
-        <v>3.666666666666667</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="E25" t="n">
         <v>3.333333333333333</v>
       </c>
       <c r="F25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G25" t="n">
         <v>4</v>
       </c>
       <c r="H25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I25" t="n">
-        <v>3.555555555555555</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="J25" t="n">
-        <v>0.6666666666666665</v>
+        <v>-0.6666666666666665</v>
       </c>
       <c r="K25" t="n">
-        <v>-0.3333333333333335</v>
+        <v>-0.6666666666666665</v>
       </c>
       <c r="L25" t="n">
-        <v>0.3333333333333335</v>
+        <v>-0.6666666666666665</v>
       </c>
     </row>
     <row r="26">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>RAFAEL ELI KATRI</t>
+          <t>PEDRO IVO AMARAL LIMA</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1491,29 +1491,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PEDRO BITTAR BARÃO</t>
+          <t>LUCAS NOVAIS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>FERNANDA DE OLIVEIRA PEREIRA</t>
+          <t>PEDRO BALBO PORTELLA</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1550,7 +1550,7 @@
         <v>3</v>
       </c>
       <c r="H28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I28" t="n">
         <v>3</v>
@@ -1562,7 +1562,7 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1571,25 +1571,39 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>LEONARDO DA FRANÇA MOURA DE ANDRADE</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+          <t>ISABELLA DOS SANTOS DE AMORIM</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" t="n">
+        <v>4</v>
+      </c>
       <c r="F29" t="n">
         <v>4</v>
       </c>
       <c r="G29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H29" t="n">
-        <v>3</v>
-      </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="I29" t="n">
+        <v>4</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -1597,25 +1611,159 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>RAFAEL COCA LEVENTHAL</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+          <t>DIOGO PEREIRA LOBO</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" t="n">
+        <v>4</v>
+      </c>
+      <c r="E30" t="n">
+        <v>4</v>
+      </c>
       <c r="F30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H30" t="n">
-        <v>3</v>
-      </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="I30" t="n">
+        <v>4</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>TALES IVALQUE TAVEIRA DE FREITAS</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" t="n">
+        <v>3</v>
+      </c>
+      <c r="H31" t="n">
+        <v>3</v>
+      </c>
+      <c r="I31" t="n">
+        <v>3</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>JULIA FIGUEIREDO</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G32" t="n">
+        <v>3</v>
+      </c>
+      <c r="H32" t="n">
+        <v>3</v>
+      </c>
+      <c r="I32" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>LUCAS HIX</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>3</v>
+      </c>
+      <c r="F33" t="n">
+        <v>3</v>
+      </c>
+      <c r="G33" t="n">
+        <v>3</v>
+      </c>
+      <c r="H33" t="n">
+        <v>3</v>
+      </c>
+      <c r="I33" t="n">
+        <v>3</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>